<commit_message>
FORM ANUGERAH template: CPH / A, B, C priced at RM7.50
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ACUVCYwJJJS64s3cKFAeYT
</commit_message>
<xml_diff>
--- a/public/templates/FORM-ANUGERAH.xlsx
+++ b/public/templates/FORM-ANUGERAH.xlsx
@@ -10829,7 +10829,7 @@
         <v>146</v>
       </c>
       <c r="B29">
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="30" spans="1:2">
@@ -10837,7 +10837,7 @@
         <v>147</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -10845,7 +10845,7 @@
         <v>148</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="32" spans="1:2">

</xml_diff>